<commit_message>
Updated to logic to include Tech, Office Work and Stockroom
</commit_message>
<xml_diff>
--- a/01_Output/Final_Allocation.xlsx
+++ b/01_Output/Final_Allocation.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H25"/>
+  <dimension ref="A1:K25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -467,6 +467,21 @@
       <c r="H1" s="1" t="inlineStr">
         <is>
           <t>SF Down</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Office Work</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Stockroom</t>
         </is>
       </c>
     </row>
@@ -487,6 +502,9 @@
       <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr"/>
       <c r="H2" t="inlineStr"/>
+      <c r="I2" t="inlineStr"/>
+      <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -505,6 +523,9 @@
       <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr"/>
       <c r="H3" t="inlineStr"/>
+      <c r="I3" t="inlineStr"/>
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -523,6 +544,9 @@
       <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr"/>
       <c r="H4" t="inlineStr"/>
+      <c r="I4" t="inlineStr"/>
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -544,17 +568,28 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>['Ricardo Gomez', 'Ethan Palmer']</t>
+          <t>['Ricardo Gomez', 'Analuisa Flores Teran']</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>['Analuisa Flores Teran', 'Finn Broderick']</t>
+          <t>['Finn Broderick']</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
           <t>['Solymar Kneale', 'Dev Mahajan']</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>['Shri Ram Gudipati']</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr"/>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>['Ethan Palmer']</t>
         </is>
       </c>
     </row>
@@ -578,17 +613,28 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>['Ricardo Gomez', 'Ethan Palmer']</t>
+          <t>['Ricardo Gomez', 'Analuisa Flores Teran']</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>['Analuisa Flores Teran', 'Finn Broderick']</t>
+          <t>['Finn Broderick']</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
           <t>['Solymar Kneale']</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>['Shri Ram Gudipati']</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr"/>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>['Ethan Palmer']</t>
         </is>
       </c>
     </row>
@@ -610,27 +656,38 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Analuisa Flores Teran</t>
+          <t>Marsailles Wesley</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>['Carson Turk', 'Marsailles Wesley']</t>
+          <t>['Carson Turk', 'Finn Broderick']</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>['Ricardo Gomez', 'Ethan Palmer']</t>
+          <t>['Ricardo Gomez', 'Analuisa Flores Teran']</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>['Finn Broderick']</t>
+          <t>[]</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>['Solymar Kneale', 'Ana* Gonzalez']</t>
+          <t>['Solymar Kneale']</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>['Shri Ram Gudipati', 'Dev Mahajan']</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr"/>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>['Ethan Palmer', 'Ana* Gonzalez']</t>
         </is>
       </c>
     </row>
@@ -647,32 +704,47 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
+          <t>Analuisa Flores Teran</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
           <t>Finn Broderick</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>Ricardo Gomez</t>
-        </is>
-      </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>['Carson Turk', 'Marsailles Wesley']</t>
+          <t>['Carson Turk', 'Josiah Galvan-Lewis']</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>['Ethan Palmer', 'Josiah Galvan-Lewis']</t>
+          <t>['Ricardo Gomez', 'Andrew (AJ) # Bowlen']</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>['Andrew (AJ) # Bowlen', 'Kaeden Stander']</t>
+          <t>['Marsailles Wesley']</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>['Ana* Gonzalez', 'Analuisa Flores Teran']</t>
+          <t>['Kaeden Stander']</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>['Shri Ram Gudipati']</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>['AJ # Alkhamees']</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>['Ethan Palmer', 'Ana* Gonzalez']</t>
         </is>
       </c>
     </row>
@@ -689,32 +761,47 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Carson Turk</t>
+          <t>Hanah # Wilkins</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Ethan Palmer</t>
+          <t>Ricardo Gomez</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>['Marsailles Wesley', 'Hanah # Wilkins']</t>
+          <t>['Carson Turk', 'Josiah Galvan-Lewis']</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>['Josiah Galvan-Lewis', 'Andrew (AJ) # Bowlen']</t>
+          <t>['Andrew (AJ) # Bowlen', 'Kevin^ Jenkins']</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>['Kaeden Stander', 'Kevin^ Jenkins']</t>
+          <t>['Marsailles Wesley']</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>['Luke* Ruhl', 'Ricardo Gomez']</t>
+          <t>['Kaeden Stander']</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>['Shri Ram Gudipati', 'Kayhaan Rashiq']</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>['AJ # Alkhamees']</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>['Ethan Palmer', 'Luke* Ruhl']</t>
         </is>
       </c>
     </row>
@@ -731,7 +818,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Marsailles Wesley</t>
+          <t>Carson Turk</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -741,22 +828,37 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>['Hanah # Wilkins', 'Kevin^ Jenkins']</t>
+          <t>['Hanah # Wilkins', 'Joaquin Mendoza']</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>['Andrew (AJ) # Bowlen', 'Carson Turk']</t>
+          <t>['Andrew (AJ) # Bowlen', 'Kevin^ Jenkins']</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>['Kaeden Stander', 'Joaquin Mendoza', 'Miguel Tanner']</t>
+          <t>['Marsailles Wesley', 'Miguel Tanner']</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>['Luke* Ruhl', 'Ricardo Gomez', 'Ethan Palmer']</t>
+          <t>['Kaeden Stander', 'Ricardo Gomez']</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>['Shri Ram Gudipati', 'Kayhaan Rashiq']</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>['AJ # Alkhamees']</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>['Ethan Palmer', 'Luke* Ruhl']</t>
         </is>
       </c>
     </row>
@@ -773,30 +875,45 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Hanah # Wilkins</t>
+          <t>Kevin^ Jenkins</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Kevin^ Jenkins</t>
+          <t>Joaquin Mendoza</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>['Josiah Galvan-Lewis', 'Elijah Kodjak']</t>
+          <t>['Hanah # Wilkins', 'Josiah Galvan-Lewis']</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>['Andrew (AJ) # Bowlen', 'Carson Turk']</t>
+          <t>['Andrew (AJ) # Bowlen', 'Elijah Kodjak']</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>['Joaquin Mendoza', 'Miguel Tanner']</t>
+          <t>['Miguel Tanner']</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
+        <is>
+          <t>['Carson Turk']</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>['Shri Ram Gudipati', 'Kayhaan Rashiq']</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>['AJ # Alkhamees']</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
         <is>
           <t>['Luke* Ruhl', 'Lauren* Koski']</t>
         </is>
@@ -820,27 +937,38 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Luke* Ruhl</t>
+          <t>Elijah Kodjak</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>['Josiah Galvan-Lewis', 'Elijah Kodjak']</t>
+          <t>['Hanah # Wilkins', 'Josiah Galvan-Lewis']</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>['Andrew (AJ) # Bowlen', 'Carson Turk']</t>
+          <t>['Andrew (AJ) # Bowlen', 'Cristian Andrade']</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>['Joaquin Mendoza', 'Cristian Andrade', 'Hanah # Wilkins']</t>
+          <t>['Kevin^ Jenkins']</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>['Lauren* Koski', 'Kevin^ Jenkins', 'Lulu (Lyndsey)* Arterburn']</t>
+          <t>['Carson Turk', 'Joaquin Mendoza']</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>['Shri Ram Gudipati', 'Kayhaan Rashiq']</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr"/>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>['Luke* Ruhl', 'Lauren* Koski', 'Lulu (Lyndsey)* Arterburn']</t>
         </is>
       </c>
     </row>
@@ -857,7 +985,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Elijah Kodjak</t>
+          <t>AJ # Alkhamees</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -867,7 +995,7 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>['Josiah Galvan-Lewis', 'Hanah # Wilkins']</t>
+          <t>['Hanah # Wilkins', 'Josiah Galvan-Lewis']</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -877,12 +1005,23 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>['AJ # Alkhamees', 'Solymar Kneale']</t>
+          <t>['Elijah Kodjak']</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>['Lulu (Lyndsey)* Arterburn', 'Joaquin Salinas']</t>
+          <t>['Solymar Kneale', 'Joaquin Salinas']</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>['Shri Ram Gudipati', 'Kayhaan Rashiq']</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr"/>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>['Lulu (Lyndsey)* Arterburn']</t>
         </is>
       </c>
     </row>
@@ -899,17 +1038,17 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Ana* Gonzalez</t>
+          <t>Scott Hackney</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Lulu (Lyndsey)* Arterburn</t>
+          <t>Mariana Cepeda</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>['Josiah Galvan-Lewis', 'Hanah # Wilkins']</t>
+          <t>['Hanah # Wilkins', 'Josiah Galvan-Lewis']</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -919,12 +1058,23 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>['AJ # Alkhamees', 'Cassidy Jacobs', 'Mariana Cepeda']</t>
+          <t>['Elijah Kodjak', 'Cristian Andrade']</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>['Scott Hackney', 'Cristian Andrade', 'Summer Sutton', 'Elijah Kodjak']</t>
+          <t>['Summer Sutton', 'AJ # Alkhamees']</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>['Shri Ram Gudipati']</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr"/>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>['Lulu (Lyndsey)* Arterburn', 'Ana* Gonzalez', 'Cassidy Jacobs']</t>
         </is>
       </c>
     </row>
@@ -941,32 +1091,43 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Cassidy Jacobs</t>
+          <t>Summer Sutton</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Mariana Cepeda</t>
+          <t>Anahi Guitierrez</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>['Josiah Galvan-Lewis', 'Hanah # Wilkins']</t>
+          <t>['Hanah # Wilkins', 'Josiah Galvan-Lewis']</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>['Anahi Guitierrez', 'Diego Navarro']</t>
+          <t>['Mariana Cepeda', 'Diego Navarro']</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>['Ana* Gonzalez', 'Lohith Ramesh', 'Saaijeesh Sottalu Naresh']</t>
+          <t>['Cristian Andrade', 'Scott Hackney']</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>['Scott Hackney', 'Cristian Andrade', 'Summer Sutton', 'Luke* Ruhl']</t>
+          <t>['Lohith Ramesh', 'Saaijeesh Sottalu Naresh']</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>['Shri Ram Gudipati']</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr"/>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>['Ana* Gonzalez', 'Cassidy Jacobs', 'Luke* Ruhl']</t>
         </is>
       </c>
     </row>
@@ -983,32 +1144,43 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Scott Hackney</t>
+          <t>Diego Navarro</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Summer Sutton</t>
+          <t>Lohith Ramesh</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>['Josiah Galvan-Lewis', 'Cassidy Jacobs']</t>
+          <t>['Josiah Galvan-Lewis', 'Cassidy Sylves']</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>['Anahi Guitierrez', 'Diego Navarro']</t>
+          <t>['Mariana Cepeda', 'Anahi Guitierrez']</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>['Ana* Gonzalez', 'Lohith Ramesh', 'Saaijeesh Sottalu Naresh']</t>
+          <t>['Scott Hackney', 'Cristian Andrade']</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>['Luke* Ruhl', 'Cristian Andrade', 'Cassidy Sylves', 'Mariana Cepeda']</t>
+          <t>['Saaijeesh Sottalu Naresh', 'Summer Sutton']</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>['Shri Ram Gudipati']</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr"/>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>['Ana* Gonzalez', 'Cassidy Jacobs', 'Luke* Ruhl']</t>
         </is>
       </c>
     </row>
@@ -1025,32 +1197,43 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Joaquin Mendoza</t>
+          <t>Saaijeesh Sottalu Naresh</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Anahi Guitierrez</t>
+          <t>Cassidy Sylves</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>['Josiah Galvan-Lewis', 'Cassidy Jacobs']</t>
+          <t>['Josiah Galvan-Lewis', 'Diego Navarro']</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>['Diego Navarro', 'Cassidy Sylves']</t>
+          <t>['Mariana Cepeda', 'Anahi Guitierrez']</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>['Ana* Gonzalez', 'Lohith Ramesh', 'Saaijeesh Sottalu Naresh']</t>
+          <t>['Scott Hackney']</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>['Mariana Cepeda', 'Scott Hackney', 'Zadie Knapp']</t>
+          <t>['Joaquin Mendoza', 'Lohith Ramesh']</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>['Shri Ram Gudipati']</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr"/>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>['Ana* Gonzalez', 'Cassidy Jacobs', 'Zadie Knapp']</t>
         </is>
       </c>
     </row>
@@ -1067,32 +1250,43 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Diego Navarro</t>
+          <t>Ana* Gonzalez</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Lohith Ramesh</t>
+          <t>Cassidy Jacobs</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>['Josiah Galvan-Lewis', 'Cassidy Jacobs']</t>
+          <t>['Josiah Galvan-Lewis', 'Diego Navarro']</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>['Cassidy Sylves', 'Serenity* Munoz']</t>
+          <t>['Mariana Cepeda', 'Anahi Guitierrez']</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>['Ana* Gonzalez', 'Saaijeesh Sottalu Naresh', 'Anahi Guitierrez']</t>
+          <t>['Saaijeesh Sottalu Naresh']</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>['Mariana Cepeda', 'Scott Hackney', 'Zadie Knapp', 'Joaquin Mendoza']</t>
+          <t>['Joaquin Mendoza', 'Lohith Ramesh']</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>['Shri Ram Gudipati']</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr"/>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>['Zadie Knapp', 'Serenity* Munoz']</t>
         </is>
       </c>
     </row>
@@ -1109,32 +1303,43 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Cassidy Sylves</t>
+          <t>Elizabeth Jurry</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Zadie Knapp</t>
+          <t>Naman Talwar</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>['Cassidy Jacobs', 'Elizabeth Jurry']</t>
+          <t>['Diego Navarro', 'Cassidy Sylves']</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>['Serenity* Munoz', 'Madelyn* Ozdarski']</t>
+          <t>['Mariana Cepeda', 'Anahi Guitierrez']</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>['Anahi Guitierrez', 'Naman Talwar']</t>
+          <t>[]</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>['Mariana Cepeda', 'Scott Hackney', 'Diego Navarro']</t>
+          <t>['Scott Hackney']</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>['Shri Ram Gudipati']</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr"/>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>['Cassidy Jacobs', 'Zadie Knapp', 'Serenity* Munoz', 'Madelyn* Ozdarski']</t>
         </is>
       </c>
     </row>
@@ -1156,27 +1361,34 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Elizabeth Jurry</t>
+          <t>Madelyn* Ozdarski</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>['Cassidy Jacobs', 'Cassidy Sylves']</t>
+          <t>['Diego Navarro', 'Cassidy Sylves']</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>['Madelyn* Ozdarski', 'Naman Talwar']</t>
+          <t>['Mariana Cepeda', 'Anahi Guitierrez']</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>['Anahi Guitierrez']</t>
+          <t>[]</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>['Mariana Cepeda', 'Diego Navarro']</t>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr"/>
+      <c r="J20" t="inlineStr"/>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>['Cassidy Jacobs']</t>
         </is>
       </c>
     </row>
@@ -1193,32 +1405,39 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Saaijeesh Sottalu Naresh</t>
+          <t>Mali Chavez</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Madelyn* Ozdarski</t>
+          <t>Aaron* Dorrance</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>['Cassidy Jacobs', 'Cassidy Sylves']</t>
+          <t>['Cassidy Sylves', 'Saaijeesh Sottalu Naresh']</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>['Naman Talwar', 'Mali Chavez']</t>
+          <t>['Elizabeth Jurry', 'Naman Talwar']</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>['Lulu (Lyndsey)* Arterburn', 'Serenity* Munoz', 'Elizabeth Jurry']</t>
+          <t>['Calvin # Levy']</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>['Aaron* Dorrance', 'Calvin # Levy', 'Ellia* Bono', 'Kayhaan Rashiq']</t>
+          <t>['Ellia* Bono', 'Kayhaan Rashiq']</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr"/>
+      <c r="J21" t="inlineStr"/>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>['Cassidy Jacobs', 'Serenity* Munoz', 'Madelyn* Ozdarski']</t>
         </is>
       </c>
     </row>
@@ -1235,32 +1454,39 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Naman Talwar</t>
+          <t>Calvin # Levy</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Aaron* Dorrance</t>
+          <t>Ellia* Bono</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>['Cassidy Jacobs', 'Cassidy Sylves']</t>
+          <t>['Cassidy Sylves', 'Saaijeesh Sottalu Naresh']</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>['Mali Chavez', 'Lulu (Lyndsey)* Arterburn']</t>
+          <t>['Elizabeth Jurry', 'Naman Talwar']</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>['Serenity* Munoz', 'Elizabeth Jurry', 'Saaijeesh Sottalu Naresh']</t>
+          <t>['Mali Chavez']</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>['Calvin # Levy', 'Ellia* Bono', 'Kayhaan Rashiq', 'Madelyn* Ozdarski']</t>
+          <t>['Kayhaan Rashiq', 'Aaron* Dorrance']</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr"/>
+      <c r="J22" t="inlineStr"/>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>['Cassidy Jacobs', 'Serenity* Munoz', 'Madelyn* Ozdarski']</t>
         </is>
       </c>
     </row>
@@ -1281,6 +1507,9 @@
       <c r="F23" t="inlineStr"/>
       <c r="G23" t="inlineStr"/>
       <c r="H23" t="inlineStr"/>
+      <c r="I23" t="inlineStr"/>
+      <c r="J23" t="inlineStr"/>
+      <c r="K23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1299,6 +1528,9 @@
       <c r="F24" t="inlineStr"/>
       <c r="G24" t="inlineStr"/>
       <c r="H24" t="inlineStr"/>
+      <c r="I24" t="inlineStr"/>
+      <c r="J24" t="inlineStr"/>
+      <c r="K24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1317,6 +1549,9 @@
       <c r="F25" t="inlineStr"/>
       <c r="G25" t="inlineStr"/>
       <c r="H25" t="inlineStr"/>
+      <c r="I25" t="inlineStr"/>
+      <c r="J25" t="inlineStr"/>
+      <c r="K25" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>